<commit_message>
Actualizacion automatica de datos - vie 22/05/2026 13:46:41,38
</commit_message>
<xml_diff>
--- a/Tareas Riesgo/Tareas de Riesgo.xlsx
+++ b/Tareas Riesgo/Tareas de Riesgo.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maria Alejandra\Downloads\Pagina Web de Riesgo VS\Tareas Riesgo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95402CD3-0705-4482-9B61-B5258FBE9A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA01970-5D01-4593-8EBF-525BD6A26FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" xr2:uid="{D78635F3-F774-46C0-9939-13AA98FCBE71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D78635F3-F774-46C0-9939-13AA98FCBE71}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$77</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -104,9 +104,6 @@
     <t>Saldos negativos</t>
   </si>
   <si>
-    <t>Revision de Billetera Usuarios - PDV</t>
-  </si>
-  <si>
     <t>Detalle de Tarea</t>
   </si>
   <si>
@@ -261,6 +258,9 @@
 • D. El Salvador: Inswitch - N1co - PayPhone - Terracal - Unlimint  
 • D. Ecuador: Englobamarketing - Inswitch - Monnet - Paycash - Unlimint  
 • Frecuencia: Diaria</t>
+  </si>
+  <si>
+    <t>Revision de Billetera Usuarios - PDV (Desfase)</t>
   </si>
 </sst>
 </file>
@@ -759,1088 +759,1084 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="150" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C77" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D77" s="1" t="s">
-        <v>62</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D76" xr:uid="{E29C3210-7A32-4834-9A63-863DBB5E8951}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D76">
-      <sortCondition ref="C2:C76"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:D77" xr:uid="{E29C3210-7A32-4834-9A63-863DBB5E8951}"/>
   <conditionalFormatting sqref="C33">
     <cfRule type="duplicateValues" dxfId="6" priority="8"/>
   </conditionalFormatting>

</xml_diff>